<commit_message>
Make hosted route planning more resilient
</commit_message>
<xml_diff>
--- a/docs/northern_states_roadtrip_attractions.xlsx
+++ b/docs/northern_states_roadtrip_attractions.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R89e4fece43274930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="Rd31fb6a7672e4d30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="Ref12a12a81c04be9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="Rdf6c686d627c49bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R0645f903a3174155"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R76d9a8851e004218"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R584cae983b804521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="Rca15b6c1039c4d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R5b58e9719dca41c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R3eebf5ec22c4492a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28586,7 +28586,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7ec3bcbc41b4272"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b4ca67370e486c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28861,7 +28861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c14e27b8cc34c69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fb58028a2584fa4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30370,7 +30370,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafc34db1c44b4c8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R969a3ef3c9614109"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30602,7 +30602,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b2730996ee04299"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b6974b585e641e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add local fallback for route start and end locations
</commit_message>
<xml_diff>
--- a/docs/northern_states_roadtrip_attractions.xlsx
+++ b/docs/northern_states_roadtrip_attractions.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R76d9a8851e004218"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R584cae983b804521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="Rca15b6c1039c4d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R5b58e9719dca41c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R3eebf5ec22c4492a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra4dc1942487a4029"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R470a5ca61c284cde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="R41bbe8f880a84178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R4e4170b0c2844115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rca2424b431d04a15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28586,7 +28586,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b4ca67370e486c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R823c2286b67f448e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28861,7 +28861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fb58028a2584fa4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe16364b09bf43d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30370,7 +30370,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R969a3ef3c9614109"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75cc5d7163e54d79"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30602,7 +30602,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b6974b585e641e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f2945a018954bdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Show route segment details on click
</commit_message>
<xml_diff>
--- a/docs/northern_states_roadtrip_attractions.xlsx
+++ b/docs/northern_states_roadtrip_attractions.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra4dc1942487a4029"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R470a5ca61c284cde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="R41bbe8f880a84178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R4e4170b0c2844115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rca2424b431d04a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd6d08eb941714c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R103370993395450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="R907f73c7f3c14d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R7f788d7d618f445d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R34298e2aef2749d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28586,7 +28586,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R823c2286b67f448e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fa17a3735304eee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28861,7 +28861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe16364b09bf43d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re128603d305d45b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30370,7 +30370,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75cc5d7163e54d79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a6d6ff34d364141"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30602,7 +30602,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f2945a018954bdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfead7bc2d2124e29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Broaden offline route location matching
</commit_message>
<xml_diff>
--- a/docs/northern_states_roadtrip_attractions.xlsx
+++ b/docs/northern_states_roadtrip_attractions.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd6d08eb941714c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R103370993395450e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="R907f73c7f3c14d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R7f788d7d618f445d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R34298e2aef2749d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1e971465dd94437a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R473715b94e4040e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="R3d638896dc2c4658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R9dcf61169a1a4898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rdebd792ffca84b32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28586,7 +28586,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fa17a3735304eee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f543839b19c4a63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28861,7 +28861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re128603d305d45b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ed19fffdc354b41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30370,7 +30370,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a6d6ff34d364141"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd92c6cfc6f554833"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30602,7 +30602,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfead7bc2d2124e29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf02e913c44544e19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use attraction dropdowns for route endpoints
</commit_message>
<xml_diff>
--- a/docs/northern_states_roadtrip_attractions.xlsx
+++ b/docs/northern_states_roadtrip_attractions.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1e971465dd94437a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R473715b94e4040e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="R3d638896dc2c4658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R9dcf61169a1a4898"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rdebd792ffca84b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rddccfcdb3db245e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R3ec5c4a65c5945e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="Rcddd7ec3495641ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="Rdf7f63aabcc649ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R2ece8a5bc10c4d1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28586,7 +28586,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f543839b19c4a63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R205e19e8e4424cba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28861,7 +28861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ed19fffdc354b41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67f52694d79e4faf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30370,7 +30370,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd92c6cfc6f554833"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra54b2840393148a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30602,7 +30602,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf02e913c44544e19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2286d6b2260f443b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add route visibility toggles
</commit_message>
<xml_diff>
--- a/docs/northern_states_roadtrip_attractions.xlsx
+++ b/docs/northern_states_roadtrip_attractions.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rddccfcdb3db245e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="R3ec5c4a65c5945e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="Rcddd7ec3495641ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="Rdf7f63aabcc649ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R2ece8a5bc10c4d1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R071edb5be89b4f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="Re803c63d570a40bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="Rb293aba0c82d4ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R6b21f159fd4146a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R4319e589509d414f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28586,7 +28586,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R205e19e8e4424cba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10041723aa7b469f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28861,7 +28861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67f52694d79e4faf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b2aa2155681435e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30370,7 +30370,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra54b2840393148a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R619307621fb04512"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30602,7 +30602,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2286d6b2260f443b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcd9250e9dfe4665"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reset saved filters for mainland USA map
</commit_message>
<xml_diff>
--- a/docs/northern_states_roadtrip_attractions.xlsx
+++ b/docs/northern_states_roadtrip_attractions.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rab308848a2834051"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="Re070df361c064db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="R805dd3cc64ee43c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R087f08f6b1684709"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R9c28be52700349c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R671abaaf31924a30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractions" sheetId="2" r:id="Reeabc3d8eeb54390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="3" r:id="R00d06415cac54f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenic Roads" sheetId="4" r:id="R3c580ea6fe5f49ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R9d5c07ab98fc41d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -33701,7 +33701,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4752d037a064f10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7248488ab5ec4e65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34410,7 +34410,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b2d0da9e2fe4355"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbe9c8996bdc41f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35919,7 +35919,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe9dd202580b483c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a5495ebbb28406c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36399,7 +36399,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21e3607099394bd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R383bc2ec35b54cbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>